<commit_message>
feat: enhance invoice fields, template, translations, and migrations
- add GST, WSBC, and GST/HST account number fields
- update invoice form, admin, views, validation, and autofill logic
- update invoice UI styles and input formatting
- update Excel invoice template and calculation logic
- add Ukrainian translations for new invoice fields
- add display order autofill logic to main admin
- squash and clean up application migrations
</commit_message>
<xml_diff>
--- a/account/invoice_templates/simple-invoice.xlsx
+++ b/account/invoice_templates/simple-invoice.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14040" windowHeight="6156"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14040" windowHeight="6150"/>
   </bookViews>
   <sheets>
     <sheet name="Invoice" sheetId="20" r:id="rId1"/>
@@ -154,10 +154,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
-    <numFmt numFmtId="168" formatCode="dd\.mm\.yyyy"/>
-    <numFmt numFmtId="169" formatCode="&quot;$&quot;#\ ##0.00_);[Red]\(&quot;$&quot;#\ ##0.00\)"/>
-    <numFmt numFmtId="170" formatCode="_(* #\ ##0.00_);_(* \(#\ ##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="171" formatCode="_(&quot;$&quot;* #\ ##0.00_);_(&quot;$&quot;* \(#\ ##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#\ ##0.00_);[Red]\(&quot;$&quot;#\ ##0.00\)"/>
+    <numFmt numFmtId="166" formatCode="_(* #\ ##0.00_);_(* \(#\ ##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_(&quot;$&quot;* #\ ##0.00_);_(&quot;$&quot;* \(#\ ##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="29">
     <font>
@@ -570,7 +570,7 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="15" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -632,11 +632,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="169" fontId="16" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="16" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -645,7 +645,7 @@
     <xf numFmtId="0" fontId="24" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -660,7 +660,7 @@
     <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="171" fontId="23" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="167" fontId="23" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -674,7 +674,7 @@
     <xf numFmtId="0" fontId="18" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="171" fontId="18" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="18" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -687,7 +687,7 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="26" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="26" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -1064,18 +1064,18 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L32"/>
-  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="2.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="5.77734375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.21875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.21875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="2.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="4.21875" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.21875" style="1"/>
+    <col min="3" max="3" width="25.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="2.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="4.28515625" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.28515625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="18" customHeight="1">
@@ -1110,7 +1110,7 @@
       <c r="G3" s="20"/>
       <c r="H3" s="20"/>
     </row>
-    <row r="4" spans="1:12" s="12" customFormat="1" ht="19.95" customHeight="1">
+    <row r="4" spans="1:12" s="12" customFormat="1" ht="19.899999999999999" customHeight="1">
       <c r="A4" s="21"/>
       <c r="B4" s="22" t="s">
         <v>1</v>
@@ -1123,11 +1123,11 @@
       </c>
       <c r="G4" s="26">
         <f ca="1">TODAY()</f>
-        <v>46179</v>
+        <v>46273</v>
       </c>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:12" ht="19.95" customHeight="1">
+    <row r="5" spans="1:12" ht="19.899999999999999" customHeight="1">
       <c r="A5" s="27"/>
       <c r="B5" s="28"/>
       <c r="C5" s="23"/>
@@ -1137,7 +1137,7 @@
       <c r="G5" s="27"/>
       <c r="H5" s="27"/>
     </row>
-    <row r="6" spans="1:12" ht="19.95" customHeight="1">
+    <row r="6" spans="1:12" ht="19.899999999999999" customHeight="1">
       <c r="A6" s="27"/>
       <c r="B6" s="30" t="s">
         <v>3</v>
@@ -1156,7 +1156,7 @@
       <c r="K6" s="64"/>
       <c r="L6" s="64"/>
     </row>
-    <row r="7" spans="1:12" ht="19.95" customHeight="1">
+    <row r="7" spans="1:12" ht="19.899999999999999" customHeight="1">
       <c r="A7" s="27"/>
       <c r="B7" s="35" t="s">
         <v>6</v>
@@ -1175,7 +1175,7 @@
       <c r="K7" s="66"/>
       <c r="L7" s="64"/>
     </row>
-    <row r="8" spans="1:12" ht="19.95" customHeight="1">
+    <row r="8" spans="1:12" ht="19.899999999999999" customHeight="1">
       <c r="A8" s="27"/>
       <c r="B8" s="36"/>
       <c r="C8" s="32"/>
@@ -1190,7 +1190,7 @@
       <c r="K8" s="68"/>
       <c r="L8" s="64"/>
     </row>
-    <row r="9" spans="1:12" ht="19.95" customHeight="1">
+    <row r="9" spans="1:12" ht="19.899999999999999" customHeight="1">
       <c r="A9" s="27"/>
       <c r="B9" s="36"/>
       <c r="C9" s="32"/>
@@ -1205,7 +1205,7 @@
       <c r="K9" s="70"/>
       <c r="L9" s="64"/>
     </row>
-    <row r="10" spans="1:12" ht="19.95" customHeight="1">
+    <row r="10" spans="1:12" ht="19.899999999999999" customHeight="1">
       <c r="A10" s="27"/>
       <c r="B10" s="36" t="s">
         <v>11</v>
@@ -1220,7 +1220,7 @@
       <c r="K10" s="64"/>
       <c r="L10" s="64"/>
     </row>
-    <row r="11" spans="1:12" ht="19.95" customHeight="1">
+    <row r="11" spans="1:12" ht="19.899999999999999" customHeight="1">
       <c r="A11" s="27"/>
       <c r="B11" s="37"/>
       <c r="C11" s="32"/>
@@ -1446,10 +1446,7 @@
       <c r="F27" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="G27" s="57">
-        <f>G26*0</f>
-        <v>0</v>
-      </c>
+      <c r="G27" s="57"/>
       <c r="H27" s="58"/>
     </row>
     <row r="28" spans="1:8" ht="19.5" customHeight="1">
@@ -1459,10 +1456,7 @@
       <c r="F28" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="G28" s="57">
-        <f>G26*0.0282</f>
-        <v>0</v>
-      </c>
+      <c r="G28" s="57"/>
       <c r="H28" s="58"/>
     </row>
     <row r="29" spans="1:8" ht="19.5" customHeight="1">
@@ -1517,25 +1511,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
     <col min="2" max="2" width="76" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="31.95" customHeight="1">
+    <row r="1" spans="1:3" ht="31.9" customHeight="1">
       <c r="A1" s="2"/>
       <c r="B1" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C1" s="4"/>
     </row>
-    <row r="2" spans="1:3" ht="16.2">
+    <row r="2" spans="1:3" ht="16.5">
       <c r="A2" s="2"/>
       <c r="B2" s="5"/>
       <c r="C2" s="4"/>
     </row>
-    <row r="3" spans="1:3" ht="16.2">
+    <row r="3" spans="1:3" ht="16.5">
       <c r="A3" s="2"/>
       <c r="B3" s="6" t="s">
         <v>22</v>
@@ -1549,79 +1543,79 @@
       </c>
       <c r="C4" s="4"/>
     </row>
-    <row r="5" spans="1:3" ht="16.2">
+    <row r="5" spans="1:3" ht="16.5">
       <c r="A5" s="2"/>
       <c r="B5" s="8"/>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:3" ht="16.2">
+    <row r="6" spans="1:3" ht="16.5">
       <c r="A6" s="2"/>
       <c r="B6" s="9" t="s">
         <v>24</v>
       </c>
       <c r="C6" s="4"/>
     </row>
-    <row r="7" spans="1:3" ht="16.2">
+    <row r="7" spans="1:3" ht="16.5">
       <c r="A7" s="2"/>
       <c r="B7" s="8"/>
       <c r="C7" s="4"/>
     </row>
-    <row r="8" spans="1:3" ht="46.2">
+    <row r="8" spans="1:3" ht="46.5">
       <c r="A8" s="2"/>
       <c r="B8" s="8" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:3" ht="16.2">
+    <row r="9" spans="1:3" ht="16.5">
       <c r="A9" s="2"/>
       <c r="B9" s="8"/>
       <c r="C9" s="4"/>
     </row>
-    <row r="10" spans="1:3" ht="31.2">
+    <row r="10" spans="1:3" ht="31.5">
       <c r="A10" s="2"/>
       <c r="B10" s="8" t="s">
         <v>26</v>
       </c>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:3" ht="16.2">
+    <row r="11" spans="1:3" ht="16.5">
       <c r="A11" s="2"/>
       <c r="B11" s="8"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:3" ht="31.2">
+    <row r="12" spans="1:3" ht="31.5">
       <c r="A12" s="2"/>
       <c r="B12" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:3" ht="16.2">
+    <row r="13" spans="1:3" ht="16.5">
       <c r="A13" s="2"/>
       <c r="B13" s="8"/>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:3" ht="16.2">
+    <row r="14" spans="1:3" ht="16.5">
       <c r="A14" s="2"/>
       <c r="B14" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:3" ht="16.2">
+    <row r="15" spans="1:3" ht="16.5">
       <c r="A15" s="2"/>
       <c r="B15" s="8" t="s">
         <v>29</v>
       </c>
       <c r="C15" s="4"/>
     </row>
-    <row r="16" spans="1:3" ht="16.2">
+    <row r="16" spans="1:3" ht="16.5">
       <c r="A16" s="2"/>
       <c r="B16" s="11"/>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:3" ht="31.8">
+    <row r="17" spans="1:3" ht="32.25">
       <c r="A17" s="2"/>
       <c r="B17" s="8" t="s">
         <v>30</v>

</xml_diff>